<commit_message>
Update industry pages workbook: add 6 new pages, drop incorporated contractor page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xNLXB75gm5xX2d5TYk2jJ
</commit_message>
<xml_diff>
--- a/exports/gondaliya-industry-pages.xlsx
+++ b/exports/gondaliya-industry-pages.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Industry Pages" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Industry Pages'!$A$1:$B$367</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Industry Pages'!$A$1:$B$368</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B367"/>
+  <dimension ref="A1:B368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1849,3005 +1849,3017 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Engineering Consultants</t>
+          <t>Employment Agencies</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-engineering-consultants/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-employment-agencies/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Environmental Consultants</t>
+          <t>Engineering Consultants</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-environmental-consultants/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-engineering-consultants/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Equipment Finance Companies</t>
+          <t>Environmental Consultants</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-equipment-finance-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-environmental-consultants/</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Escape Rooms</t>
+          <t>Equipment Finance Companies</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-escape-rooms/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-equipment-finance-companies/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Esports Organizations</t>
+          <t>Escape Rooms</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-esports-organizations/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-escape-rooms/</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Ethnic Food Stores</t>
+          <t>Esports Organizations</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-ethnic-food-stores/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-esports-organizations/</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Event Venues</t>
+          <t>Ethnic Food Stores</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-event-venues/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-ethnic-food-stores/</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Excavation Companies</t>
+          <t>Event Venues</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-excavation-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-event-venues/</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Executive Coaches</t>
+          <t>Excavation Companies</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-executive-coaches/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-excavation-companies/</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Exporters</t>
+          <t>Executive Coaches</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-exporters/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-executive-coaches/</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Factoring Companies</t>
+          <t>Exporters</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-factoring-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-exporters/</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Family Doctors</t>
+          <t>Factoring Companies</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-family-doctors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-factoring-companies/</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Family Entertainment Centres</t>
+          <t>Family Doctors</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-family-entertainment-centres/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-family-doctors/</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Family-Owned Businesses</t>
+          <t>Family Entertainment Centres</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-family-owned-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-family-entertainment-centres/</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Farmland Investors</t>
+          <t>Family-Owned Businesses</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-farmland-investors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-family-owned-businesses/</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Farms</t>
+          <t>Farmland Investors</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-farms/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-farmland-investors/</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Fencing and Deck Builders</t>
+          <t>Farms</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-fencing-and-deck-builders/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-farms/</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Fertility Clinics</t>
+          <t>Fencing and Deck Builders</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-fertility-clinics/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-fencing-and-deck-builders/</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Film Production Companies</t>
+          <t>Fertility Clinics</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-film-production-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-fertility-clinics/</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Finance Contractors</t>
+          <t>Film Production Companies</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-finance-contractors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-film-production-companies/</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Fine Dining Restaurants</t>
+          <t>Finance Contractors</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-fine-dining-restaurants/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-finance-contractors/</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Fire Protection Contractors</t>
+          <t>Fine Dining Restaurants</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-fire-protection-contractors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-fine-dining-restaurants/</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Fleet Owners</t>
+          <t>Fire Protection Contractors</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-fleet-owners/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-fire-protection-contractors/</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Food &amp; Beverage Businesses</t>
+          <t>Fleet Owners</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/food-beverage-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-fleet-owners/</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Food Delivery Drivers</t>
+          <t>Food &amp; Beverage Businesses</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-food-delivery-drivers/</t>
+          <t>https://gondaliyacpa.ca/food-beverage-businesses/</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Food Franchise Store</t>
+          <t>Food Delivery Drivers</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/food-franchise-store/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-food-delivery-drivers/</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Foreign Employers Hiring in Canada</t>
+          <t>Food Franchise Store</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-foreign-employers-hiring-in-canada/</t>
+          <t>https://gondaliyacpa.ca/food-franchise-store/</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Foreign Investors in Canadian Real Estate</t>
+          <t>Foreign Employers Hiring in Canada</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-foreign-investors-in-canadian-real-estate/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-foreign-employers-hiring-in-canada/</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Foreign Shareholders of Canadian Corporations</t>
+          <t>Foreign Investors in Canadian Real Estate</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-foreign-shareholders-of-canadian-corporations/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-foreign-investors-in-canadian-real-estate/</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Forestry Companies</t>
+          <t>Foreign Shareholders of Canadian Corporations</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-forestry-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-foreign-shareholders-of-canadian-corporations/</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Franchises</t>
+          <t>Forestry Companies</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/franchise-accounting/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-forestry-companies/</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Freelance Consultants (Business/ Management)</t>
+          <t>Franchises</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/freelance-consultant-business-management/</t>
+          <t>https://gondaliyacpa.ca/franchise-accounting/</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Freight Brokers</t>
+          <t>Freelance Consultants (Business/ Management)</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-freight-brokers/</t>
+          <t>https://gondaliyacpa.ca/freelance-consultant-business-management/</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Freight Forwarders</t>
+          <t>Freight Brokers</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-freight-forwarders/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-freight-brokers/</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Fulfillment Centres</t>
+          <t>Freight Forwarders</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-fulfillment-centres/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-freight-forwarders/</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Furniture Manufacturers</t>
+          <t>Fulfillment Centres</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-furniture-manufacturers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-fulfillment-centres/</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Garage Door Companies</t>
+          <t>Furniture Manufacturers</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-garage-door-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-furniture-manufacturers/</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Grant Writing Consultants</t>
+          <t>Garage Door Companies</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-grant-writing-consultants/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-garage-door-companies/</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Graphic Design &amp; Creative Studios</t>
+          <t>Grant Writing Consultants</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/graphic-design-creative-studios/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-grant-writing-consultants/</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Green Card Holders in Canada</t>
+          <t>Graphic Design &amp; Creative Studios</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-green-card-holders-in-canada/</t>
+          <t>https://gondaliyacpa.ca/graphic-design-creative-studios/</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Grocery Stores</t>
+          <t>Green Card Holders in Canada</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/grocery-store/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-green-card-holders-in-canada/</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Gutter Cleaning Businesses</t>
+          <t>Grocery Stores</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-gutter-cleaning-businesses/</t>
+          <t>https://gondaliyacpa.ca/grocery-store/</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Gyms</t>
+          <t>Gutter Cleaning Businesses</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-gyms/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-gutter-cleaning-businesses/</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Hair Stylists</t>
+          <t>Gyms</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-hair-stylists/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-gyms/</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Handyman Businesses</t>
+          <t>Hair Stylists</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-handyman-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-hair-stylists/</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Hardware Startups</t>
+          <t>Handyman Businesses</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-hardware-startups/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-handyman-businesses/</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Health and Safety Consultants</t>
+          <t>Hardware Startups</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-health-and-safety-consultants/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-hardware-startups/</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Health and Safety Consultants</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/healthcare/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-health-and-safety-consultants/</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Healthcare Accounting &amp; Bookkeeping</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-bookkeeping-services-for-healthcare/</t>
+          <t>https://gondaliyacpa.ca/healthcare/</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Healthtech Companies</t>
+          <t>Healthcare Accounting &amp; Bookkeeping</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-healthtech-companies/</t>
+          <t>https://gondaliyacpa.ca/accounting-bookkeeping-services-for-healthcare/</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Heavy Equipment Operators</t>
+          <t>Healthtech Companies</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-heavy-equipment-operators/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-healthtech-companies/</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Home Stagers</t>
+          <t>Heavy Equipment Operators</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-home-stagers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-heavy-equipment-operators/</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Home-Based Businesses</t>
+          <t>Home Stagers</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-home-based-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-home-stagers/</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Hotel and Motel</t>
+          <t>Home-Based Businesses</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/hotel-and-motel/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-home-based-businesses/</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>House Flippers</t>
+          <t>Hotel and Motel</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-house-flippers/</t>
+          <t>https://gondaliyacpa.ca/hotel-and-motel/</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>HVAC Contractors</t>
+          <t>House Flippers</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-hvac-contractors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-house-flippers/</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Ice Cream Shops</t>
+          <t>Human Resources Consultants</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-ice-cream-shops/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-human-resources-consultants/</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Immigrants with Foreign Assets</t>
+          <t>HVAC Contractors</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-immigrants-with-foreign-assets/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-hvac-contractors/</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Immigration Consultants</t>
+          <t>Ice Cream Shops</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-immigration-consultants/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-ice-cream-shops/</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Import Export</t>
+          <t>Immigrants with Foreign Assets</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/import-export-accounting/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-immigrants-with-foreign-assets/</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Importers</t>
+          <t>Immigration Consultants</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-importers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-immigration-consultants/</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Incorporated Businesses</t>
+          <t>Import Export</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-incorporated-businesses/</t>
+          <t>https://gondaliyacpa.ca/import-export-accounting/</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Incorporated Contractors</t>
+          <t>Importers</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/incorporated-contractor-accountant-toronto/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-importers/</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Industrial Manufacturers</t>
+          <t>Incorporated Businesses</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-industrial-manufacturers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-incorporated-businesses/</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Insulation Contractors</t>
+          <t>Industrial Manufacturers</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-insulation-contractors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-industrial-manufacturers/</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Insurance Agents</t>
+          <t>Insulation Contractors</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-insurance-agents/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-insulation-contractors/</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Insurance Brokers</t>
+          <t>Insurance Agents</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-insurance-brokers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-insurance-agents/</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Interior Designers</t>
+          <t>Insurance Brokers</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-interior-designers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-insurance-brokers/</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Interlocking and Hardscape Contractors</t>
+          <t>Interior Designers</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-interlocking-and-hardscape-contractors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-interior-designers/</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>International Students with Businesses</t>
+          <t>Interlocking and Hardscape Contractors</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-international-students-with-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-interlocking-and-hardscape-contractors/</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Investment Corporations</t>
+          <t>International Students with Businesses</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-investment-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-international-students-with-businesses/</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Investment Holding &amp; Investment Companies</t>
+          <t>Investment Corporations</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/investment-holding-investment-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-investment-companies/</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>IT Contractors</t>
+          <t>Investment Holding &amp; Investment Companies</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-it-contractors/</t>
+          <t>https://gondaliyacpa.ca/investment-holding-investment-companies/</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>IT Staffing Companies</t>
+          <t>IT Contractors</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-it-staffing-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-it-contractors/</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>IT Support &amp; Web Development</t>
+          <t>IT Staffing Companies</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/it-support-web-development/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-it-staffing-companies/</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Joint Venture Businesses</t>
+          <t>IT Support &amp; Web Development</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-joint-venture-businesses/</t>
+          <t>https://gondaliyacpa.ca/it-support-web-development/</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Land Surveying Companies</t>
+          <t>Joint Venture Businesses</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-land-surveying-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-joint-venture-businesses/</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Landscaping Companies</t>
+          <t>Land Surveying Companies</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-landscaping-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-land-surveying-companies/</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Lash and Brow Studios</t>
+          <t>Landscaping Companies</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-lash-and-brow-studios/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-landscaping-companies/</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Last-Mile Delivery Businesses</t>
+          <t>Lash and Brow Studios</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-last-mile-delivery-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-lash-and-brow-studios/</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Laundry Businesses</t>
+          <t>Last-Mile Delivery Businesses</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-laundry-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-last-mile-delivery-businesses/</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Lawn Care Businesses</t>
+          <t>Laundry Businesses</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-lawn-care-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-laundry-businesses/</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Lawyers &amp; Law Firms</t>
+          <t>Lawn Care Businesses</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/lawyers-law-firms/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-lawn-care-businesses/</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Leasing Companies</t>
+          <t>Lawyers &amp; Law Firms</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-leasing-companies/</t>
+          <t>https://gondaliyacpa.ca/lawyers-law-firms/</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Limousine Companies</t>
+          <t>Leasing Companies</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-limousine-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-leasing-companies/</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Locksmiths</t>
+          <t>Limousine Companies</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-locksmiths/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-limousine-companies/</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Makeup Artists</t>
+          <t>Locksmiths</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-makeup-artists/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-locksmiths/</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Managed Service Providers</t>
+          <t>Makeup Artists</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-managed-service-providers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-makeup-artists/</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Managed Service Providers</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/manufacturing/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-managed-service-providers/</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Marine Repair Businesses</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-marine-repair-businesses/</t>
+          <t>https://gondaliyacpa.ca/manufacturing/</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Market Research Firms</t>
+          <t>Marine Repair Businesses</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-market-research-firms/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-marine-repair-businesses/</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Marketing, Advertising &amp; PR Agencies</t>
+          <t>Market Research Firms</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/marketing-advertising-pr-agencies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-market-research-firms/</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Martial Arts Schools</t>
+          <t>Marketing, Advertising &amp; PR Agencies</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-martial-arts-schools/</t>
+          <t>https://gondaliyacpa.ca/marketing-advertising-pr-agencies/</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Masonry Contractors</t>
+          <t>Martial Arts Schools</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-masonry-contractors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-martial-arts-schools/</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Mechanics</t>
+          <t>Masonry Contractors</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-mechanics/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-masonry-contractors/</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Medical Clinics</t>
+          <t>Mechanics</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/medical-clinic-accounting/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-mechanics/</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Medical Device Distributors</t>
+          <t>Medical Clinics</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-medical-device-distributors/</t>
+          <t>https://gondaliyacpa.ca/medical-clinic-accounting/</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Medium-Sized Businesses</t>
+          <t>Medical Device Distributors</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-services-for-medium-sized-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-medical-device-distributors/</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Millwork Companies</t>
+          <t>Medium-Sized Businesses</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-millwork-companies/</t>
+          <t>https://gondaliyacpa.ca/accounting-services-for-medium-sized-businesses/</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Mining Companies</t>
+          <t>Millwork Companies</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-mining-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-millwork-companies/</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Money Service Businesses</t>
+          <t>Mining Companies</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-money-service-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-mining-companies/</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Mortgage Brokers</t>
+          <t>Money Service Businesses</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/mortgage-brokers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-money-service-businesses/</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Motorcycle Dealers</t>
+          <t>Mortgage Brokers</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-motorcycle-dealers/</t>
+          <t>https://gondaliyacpa.ca/mortgage-brokers/</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Movie Theatres</t>
+          <t>Motorcycle Dealers</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-movie-theatres/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-motorcycle-dealers/</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Moving Companies</t>
+          <t>Movie Theatres</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-moving-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-movie-theatres/</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Multi-Residential Building Owners</t>
+          <t>Moving Companies</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-multi-residential-building-owners/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-moving-companies/</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Music Producers</t>
+          <t>Multi-Residential Building Owners</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-music-producers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-multi-residential-building-owners/</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Musicians</t>
+          <t>Music Producers</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-musicians/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-music-producers/</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Mutual Fund Representatives</t>
+          <t>Musicians</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-mutual-fund-representatives/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-musicians/</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Nail Salons</t>
+          <t>Mutual Fund Representatives</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-nail-salons/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-mutual-fund-representatives/</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Newcomer Business Owners</t>
+          <t>Nail Salons</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-newcomer-business-owners/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-nail-salons/</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Nightclubs</t>
+          <t>Newcomer Business Owners</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-nightclubs/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-newcomer-business-owners/</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>No-Code Development Agencies</t>
+          <t>Nightclubs</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-no-code-development-agencies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-nightclubs/</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Notaries</t>
+          <t>No-Code Development Agencies</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-notaries/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-no-code-development-agencies/</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Numbered Companies</t>
+          <t>Notaries</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-numbered-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-notaries/</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Nurses</t>
+          <t>Numbered Companies</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-nurses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-numbered-companies/</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Nutritionists</t>
+          <t>Nurses</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-nutritionists/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-nurses/</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Occupational Therapists</t>
+          <t>Nutritionists</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-occupational-therapists/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-nutritionists/</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Oil and Gas Companies</t>
+          <t>Occupational Therapists</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-oil-and-gas-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-occupational-therapists/</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Online Course Creators</t>
+          <t>Oil and Gas Companies</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-online-course-creators/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-oil-and-gas-companies/</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Online Education Businesses</t>
+          <t>Online Course Creators</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-online-education-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-online-course-creators/</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Online Grocery Businesses</t>
+          <t>Online Education Businesses</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-online-grocery-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-online-education-businesses/</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Online Resellers</t>
+          <t>Online Grocery Businesses</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-online-resellers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-online-grocery-businesses/</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>OnlyFans Creators</t>
+          <t>Online Resellers</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/onlyfans-creators-taxes-for-canadians/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-online-resellers/</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Optometrists</t>
+          <t>OnlyFans Creators</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-optometrists/</t>
+          <t>https://gondaliyacpa.ca/onlyfans-creators-taxes-for-canadians/</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Osteopaths</t>
+          <t>Optometrists</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-osteopaths/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-optometrists/</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Parking Lot Businesses</t>
+          <t>Osteopaths</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-parking-lot-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-osteopaths/</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Partnerships</t>
+          <t>Parking Lot Businesses</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-partnerships/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-parking-lot-businesses/</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Party Rental Businesses</t>
+          <t>Partnerships</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-party-rental-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-partnerships/</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Paving Companies</t>
+          <t>Party Rental Businesses</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-paving-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-party-rental-businesses/</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Pawn Shops</t>
+          <t>Paving Companies</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-pawn-shops/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-paving-companies/</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Performing Arts Companies</t>
+          <t>Pawn Shops</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-performing-arts-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-pawn-shops/</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Personal Support Worker Businesses</t>
+          <t>Performing Arts Companies</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-personal-support-worker-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-performing-arts-companies/</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Personal Trainers &amp; Fitness Businesses</t>
+          <t>Personal Support Worker Businesses</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/personal-trainers-fitness-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-personal-support-worker-businesses/</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Pet Boarding Businesses</t>
+          <t>Personal Trainers &amp; Fitness Businesses</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-pet-boarding-businesses/</t>
+          <t>https://gondaliyacpa.ca/personal-trainers-fitness-businesses/</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Pet Grooming Businesses</t>
+          <t>Pet Boarding Businesses</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-pet-grooming-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-pet-boarding-businesses/</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Pet Sitting Businesses</t>
+          <t>Pet Grooming Businesses</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-pet-sitting-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-pet-grooming-businesses/</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Pharmacies</t>
+          <t>Pet Sitting Businesses</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/pharmacies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-pet-sitting-businesses/</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Photo Booth Businesses</t>
+          <t>Pharmacies</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-photo-booth-businesses/</t>
+          <t>https://gondaliyacpa.ca/pharmacies/</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography</t>
+          <t>Photo Booth Businesses</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/photography-videography/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-photo-booth-businesses/</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Pilates Studios</t>
+          <t>Photography &amp; Videography</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-pilates-studios/</t>
+          <t>https://gondaliyacpa.ca/photography-videography/</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Pizzerias</t>
+          <t>Pilates Studios</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-pizzerias/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-pilates-studios/</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Plumbers</t>
+          <t>Pizzerias</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-plumbers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-pizzerias/</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Portable Toilet Rental Businesses</t>
+          <t>Plumbers</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-portable-toilet-rental-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-plumbers/</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Portfolio Managers</t>
+          <t>Portable Toilet Rental Businesses</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-portfolio-managers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-portable-toilet-rental-businesses/</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Powersports Dealers</t>
+          <t>Portfolio Managers</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-powersports-dealers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-portfolio-managers/</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Pre-Construction Condo Investors &amp; Flips</t>
+          <t>Powersports Dealers</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/pre-construction-condo-investors-flips/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-powersports-dealers/</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Pressure Washing Businesses</t>
+          <t>Pre-Construction Condo Investors &amp; Flips</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-pressure-washing-businesses/</t>
+          <t>https://gondaliyacpa.ca/pre-construction-condo-investors-flips/</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Print-on-Demand Businesses</t>
+          <t>Pressure Washing Businesses</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-print-on-demand-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-pressure-washing-businesses/</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Private Equity Firms</t>
+          <t>Print-on-Demand Businesses</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-private-equity-firms/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-print-on-demand-businesses/</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Private Investigators</t>
+          <t>Private Equity Firms</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-private-investigators/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-private-equity-firms/</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Private Lenders</t>
+          <t>Private Investigators</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-private-lenders/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-private-investigators/</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Product Design Studios</t>
+          <t>Private Lenders</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-product-design-studios/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-private-lenders/</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Professional Service Consultants</t>
+          <t>Product Design Studios</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/professional-service-consultants/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-product-design-studios/</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Property Developers &amp; Builders</t>
+          <t>Professional Service Consultants</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/property-developers-builders/</t>
+          <t>https://gondaliyacpa.ca/professional-service-consultants/</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Property Management Companies</t>
+          <t>Property Developers &amp; Builders</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/property-management-companies/</t>
+          <t>https://gondaliyacpa.ca/property-developers-builders/</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Psychologists, Psychotherapists &amp; Mental Health Professionals</t>
+          <t>Property Management Companies</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/psychologists-psychotherapists-mental-health-professionals/</t>
+          <t>https://gondaliyacpa.ca/property-management-companies/</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Public Speakers</t>
+          <t>Psychologists, Psychotherapists &amp; Mental Health Professionals</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-public-speakers/</t>
+          <t>https://gondaliyacpa.ca/psychologists-psychotherapists-mental-health-professionals/</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Publishers</t>
+          <t>Public Speakers</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-publishers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-public-speakers/</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Pubs</t>
+          <t>Publishers</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-pubs/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-publishers/</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Real Estate Agents, Realtors &amp; Brokerages</t>
+          <t>Pubs</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/real-estate-agents-realtors-brokerages/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-pubs/</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Real Estate Investors</t>
+          <t>Real Estate Agents, Realtors &amp; Brokerages</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/real-estate-accountant/</t>
+          <t>https://gondaliyacpa.ca/real-estate-agents-realtors-brokerages/</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Real Estate Syndicators</t>
+          <t>Real Estate Investors</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-real-estate-syndicators/</t>
+          <t>https://gondaliyacpa.ca/real-estate-accountant/</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Recording Studios</t>
+          <t>Real Estate Syndicators</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-recording-studios/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-real-estate-syndicators/</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Recycling Companies</t>
+          <t>Recording Studios</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-recycling-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-recording-studios/</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Rental Property Owners</t>
+          <t>Recycling Companies</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-rental-property-owners/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-recycling-companies/</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Residential &amp; Commercial Cleaning</t>
+          <t>Rental Property Owners</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/residential-commercial-cleaning/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-rental-property-owners/</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Restaurant Accounting &amp; Bookkeeping</t>
+          <t>Residential &amp; Commercial Cleaning</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-and-bookkeeping-services-for-restaurants/</t>
+          <t>https://gondaliyacpa.ca/residential-commercial-cleaning/</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Restaurant Franchisees</t>
+          <t>Restaurant Accounting &amp; Bookkeeping</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-restaurant-franchisees/</t>
+          <t>https://gondaliyacpa.ca/accounting-and-bookkeeping-services-for-restaurants/</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Restaurants</t>
+          <t>Restaurant Franchisees</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/restaurants/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-restaurant-franchisees/</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Restoration Companies</t>
+          <t>Restaurants</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-restoration-companies/</t>
+          <t>https://gondaliyacpa.ca/restaurants/</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Retail &amp; Consumer Goods Businesses</t>
+          <t>Restoration Companies</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/retail-consumer-goods-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-restoration-companies/</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Retirement Homes</t>
+          <t>Retail &amp; Consumer Goods Businesses</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-retirement-homes/</t>
+          <t>https://gondaliyacpa.ca/retail-consumer-goods-businesses/</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Rideshare Drivers</t>
+          <t>Retirement Homes</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-rideshare-drivers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-retirement-homes/</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>RV Dealers</t>
+          <t>Rideshare Drivers</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-rv-dealers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-rideshare-drivers/</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>RV Parks</t>
+          <t>RV Dealers</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-rv-parks/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-rv-dealers/</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Sawmills</t>
+          <t>RV Parks</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-sawmills/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-rv-parks/</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Scaffolding Companies</t>
+          <t>Sawmills</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-scaffolding-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-sawmills/</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Scale-Up Companies</t>
+          <t>Scaffolding Companies</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-scale-up-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-scaffolding-companies/</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>School Bus Operators</t>
+          <t>Scale-Up Companies</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-school-bus-operators/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-scale-up-companies/</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Second-Generation Family Businesses</t>
+          <t>School Bus Operators</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-second-generation-family-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-school-bus-operators/</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Security Companies</t>
+          <t>Second-Generation Family Businesses</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-security-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-second-generation-family-businesses/</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Security Guard Companies</t>
+          <t>Security Companies</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-security-guard-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-security-companies/</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Self Employed</t>
+          <t>Security Guard Companies</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/self-employed-accountant/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-security-guard-companies/</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Shoe Stores</t>
+          <t>Self Employed</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-shoe-stores/</t>
+          <t>https://gondaliyacpa.ca/self-employed-accountant/</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Shopify Accounting and Bookkeeping</t>
+          <t>Shoe Stores</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/shopify-accounting-and-bookkeeping/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-shoe-stores/</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Side-Hustle Businesses</t>
+          <t>Shopify Accounting and Bookkeeping</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-side-hustle-businesses/</t>
+          <t>https://gondaliyacpa.ca/shopify-accounting-and-bookkeeping/</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Sign Installation Companies</t>
+          <t>Side-Hustle Businesses</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-sign-installation-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-side-hustle-businesses/</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Ski Resorts</t>
+          <t>Sign Installation Companies</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-ski-resorts/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-sign-installation-companies/</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Skill Trades</t>
+          <t>Ski Resorts</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/skilled-trades/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-ski-resorts/</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Sleep Clinics</t>
+          <t>Skill Trades</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-sleep-clinics/</t>
+          <t>https://gondaliyacpa.ca/skilled-trades/</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Small Business Accounting Services</t>
+          <t>Sleep Clinics</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/small-business-accounting-services/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-sleep-clinics/</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Small Business Tax Services</t>
+          <t>Small Business Accounting Services</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-and-tax-services-for-small-businesses/</t>
+          <t>https://gondaliyacpa.ca/small-business-accounting-services/</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Small Businesses</t>
+          <t>Small Business Tax Services</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/small-business-accountant/</t>
+          <t>https://gondaliyacpa.ca/accounting-and-tax-services-for-small-businesses/</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Small Engine Repair Businesses</t>
+          <t>Small Businesses</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-small-engine-repair-businesses/</t>
+          <t>https://gondaliyacpa.ca/small-business-accountant/</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Snow Removal Businesses</t>
+          <t>Small Engine Repair Businesses</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-snow-removal-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-small-engine-repair-businesses/</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Snowbirds</t>
+          <t>Snow Removal Businesses</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-snowbirds/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-snow-removal-businesses/</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Software Companies</t>
+          <t>Snowbirds</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-for-software-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-snowbirds/</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Software Development &amp; IT Consultants</t>
+          <t>Software Companies</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/software-development-it-consultants/</t>
+          <t>https://gondaliyacpa.ca/accounting-for-software-companies/</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Software Resellers</t>
+          <t>Software Development &amp; IT Consultants</t>
         </is>
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-software-resellers/</t>
+          <t>https://gondaliyacpa.ca/software-development-it-consultants/</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Solar Installation Companies</t>
+          <t>Software Resellers</t>
         </is>
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-solar-installation-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-software-resellers/</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Sole Proprietors</t>
+          <t>Solar Installation Companies</t>
         </is>
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-sole-proprietors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-solar-installation-companies/</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Spas and Wellness Clinics</t>
+          <t>Sole Proprietors</t>
         </is>
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/spas-wellness-clinic/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-sole-proprietors/</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Specialist Physicians</t>
+          <t>Spas and Wellness Clinics</t>
         </is>
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-specialist-physicians/</t>
+          <t>https://gondaliyacpa.ca/spas-wellness-clinic/</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Specialized Haulers</t>
+          <t>Specialist Physicians</t>
         </is>
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-specialized-haulers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-specialist-physicians/</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Speech-Language Pathologists</t>
+          <t>Specialized Haulers</t>
         </is>
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-speech-language-pathologists/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-specialized-haulers/</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Sports Leagues</t>
+          <t>Speech-Language Pathologists</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-sports-leagues/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-speech-language-pathologists/</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Staffing Agencies</t>
+          <t>Sports Leagues</t>
         </is>
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-staffing-agencies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-sports-leagues/</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Startup Accounting &amp; Bookkeeping</t>
+          <t>Staffing Agencies</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-and-bookkeeping-services-for-startups/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-staffing-agencies/</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Startups</t>
+          <t>Startup Accounting &amp; Bookkeeping</t>
         </is>
       </c>
       <c r="B327" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-for-startups/</t>
+          <t>https://gondaliyacpa.ca/accounting-and-bookkeeping-services-for-startups/</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Storage Facility Owners</t>
+          <t>Startups</t>
         </is>
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-storage-facility-owners/</t>
+          <t>https://gondaliyacpa.ca/accounting-for-startups/</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>Student Rental Owners</t>
+          <t>Storage Facility Owners</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-student-rental-owners/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-storage-facility-owners/</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Subscription Box Businesses</t>
+          <t>Student Rental Owners</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-subscription-box-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-student-rental-owners/</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Summer Camps</t>
+          <t>Subscription Box Businesses</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-summer-camps/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-subscription-box-businesses/</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Supplement Brands</t>
+          <t>Summer Camps</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-supplement-brands/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-summer-camps/</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Taxi Businesses</t>
+          <t>Supplement Brands</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-taxi-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-supplement-brands/</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Tech Companies</t>
+          <t>Taxi Businesses</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/tech-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-taxi-businesses/</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Technology &amp; Communications Companies</t>
+          <t>Tech Companies</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/technology-communications-companies/</t>
+          <t>https://gondaliyacpa.ca/tech-companies/</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Technology Company Accounting &amp; Bookkeeping</t>
+          <t>Technology &amp; Communications Companies</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-and-bookkeeping-services-for-technology-companies/</t>
+          <t>https://gondaliyacpa.ca/technology-communications-companies/</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Technology Startups &amp; SaaS Companies</t>
+          <t>Technology Company Accounting &amp; Bookkeeping</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/technology-startups-saas-companies/</t>
+          <t>https://gondaliyacpa.ca/accounting-and-bookkeeping-services-for-technology-companies/</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Third-Party Logistics Providers</t>
+          <t>Technology Startups &amp; SaaS Companies</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-third-party-logistics-providers/</t>
+          <t>https://gondaliyacpa.ca/technology-startups-saas-companies/</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Tire Shops</t>
+          <t>Third-Party Logistics Providers</t>
         </is>
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-tire-shops/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-third-party-logistics-providers/</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Tour Operators</t>
+          <t>Tire Shops</t>
         </is>
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-tour-operators/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-tire-shops/</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Towing Companies</t>
+          <t>Tour Operators</t>
         </is>
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-towing-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-tour-operators/</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Toy Stores</t>
+          <t>Towing Companies</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-toy-stores/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-towing-companies/</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Trade Schools</t>
+          <t>Toy Stores</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-trade-schools/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-toy-stores/</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Translation Services</t>
+          <t>Trade Schools</t>
         </is>
       </c>
       <c r="B344" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-translation-services/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-trade-schools/</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Transportation &amp; Logistics Companies</t>
+          <t>Translation Services</t>
         </is>
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/transportation-logistics-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-translation-services/</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Travel Agencies</t>
+          <t>Transportation &amp; Logistics Companies</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-travel-agencies/</t>
+          <t>https://gondaliyacpa.ca/transportation-logistics-companies/</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Tree Service Companies</t>
+          <t>Travel Agencies</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-tree-service-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-travel-agencies/</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Truck Dispatch Businesses</t>
+          <t>Tree Service Companies</t>
         </is>
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-truck-dispatch-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-tree-service-companies/</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Trucking</t>
+          <t>Truck Dispatch Businesses</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-truck-drivers-trucking-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-truck-dispatch-businesses/</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Trucking Accounting &amp; Bookkeeping</t>
+          <t>Trucking</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accounting-and-bookkeeping-services-for-trucking-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-truck-drivers-trucking-companies/</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Twitch Streamers</t>
+          <t>Trucking Accounting &amp; Bookkeeping</t>
         </is>
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-twitch-streamers/</t>
+          <t>https://gondaliyacpa.ca/accounting-and-bookkeeping-services-for-trucking-businesses/</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Two-Shareholder Corporations</t>
+          <t>Twitch Streamers</t>
         </is>
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-two-shareholder-corporations/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-twitch-streamers/</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>Uber Drivers</t>
+          <t>Two-Shareholder Corporations</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-uber-drivers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-two-shareholder-corporations/</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>US Citizens Living in Canada</t>
+          <t>Uber Drivers</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-us-citizens-living-in-canada/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-uber-drivers/</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>Used-Car Dealerships</t>
+          <t>US Citizens Living in Canada</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-used-car-dealerships/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-us-citizens-living-in-canada/</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>Venture Capital Firms</t>
+          <t>Used-Car Dealerships</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-venture-capital-firms/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-used-car-dealerships/</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Veterinary</t>
+          <t>Venture Capital Firms</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/veterinary/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-venture-capital-firms/</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>Virtual Assistants</t>
+          <t>Veterinary</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-virtual-assistants/</t>
+          <t>https://gondaliyacpa.ca/veterinary/</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>Walk-In Clinics</t>
+          <t>Virtual Assistants</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-walk-in-clinics/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-virtual-assistants/</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>Waste Collection Companies</t>
+          <t>Walk-In Clinics</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-waste-collection-companies/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-walk-in-clinics/</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>Waterproofing Contractors</t>
+          <t>Waste Collection Companies</t>
         </is>
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-waterproofing-contractors/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-waste-collection-companies/</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>Wedding Venues</t>
+          <t>Waterproofing Contractors</t>
         </is>
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-wedding-venues/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-waterproofing-contractors/</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Wholesale Businesses</t>
+          <t>Wedding Venues</t>
         </is>
       </c>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-wholesale-businesses/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-wedding-venues/</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>Wholesale E-Commerce Sellers</t>
+          <t>Wholesale Businesses</t>
         </is>
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-wholesale-e-commerce-sellers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-wholesale-businesses/</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>Window and Door Installers</t>
+          <t>Wholesale E-Commerce Sellers</t>
         </is>
       </c>
       <c r="B365" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/accountant-for-window-and-door-installers/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-wholesale-e-commerce-sellers/</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>WooCommerce Accounting and Bookkeeping</t>
+          <t>Window and Door Installers</t>
         </is>
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>https://gondaliyacpa.ca/woocommerce-accounting-and-bookkeeping/</t>
+          <t>https://gondaliyacpa.ca/accountant-for-window-and-door-installers/</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
+          <t>WooCommerce Accounting and Bookkeeping</t>
+        </is>
+      </c>
+      <c r="B367" s="2" t="inlineStr">
+        <is>
+          <t>https://gondaliyacpa.ca/woocommerce-accounting-and-bookkeeping/</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
           <t>Yoga Studios</t>
         </is>
       </c>
-      <c r="B367" s="2" t="inlineStr">
+      <c r="B368" s="2" t="inlineStr">
         <is>
           <t>https://gondaliyacpa.ca/accountant-for-yoga-studios/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B367"/>
+  <autoFilter ref="A1:B368"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -5215,6 +5227,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B365" r:id="rId364"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B366" r:id="rId365"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B368" r:id="rId367"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>